<commit_message>
fix: D87 amended — poster template at 34 x 22.5 in with abstract, methods, conclusions, limitations, references, acknowledgments sections and author photo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
+++ b/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Title · The question and what it adds</t>
+          <t>Title · Abstract · The question and why it matters · What is already known</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -644,7 +644,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Checks and verification · verification status line</t>
+          <t>Methods · Checks and verification · verification status line</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -724,7 +724,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Headline · What this means, and where it stops</t>
+          <t>Headline · Conclusions · Limitations</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Sources, AI use, and credits</t>
+          <t>AI use disclosure · References · Acknowledgments</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>9–10 pts: A clear reading order: the finding is found in seconds, and the question, result, and boundary in a ninety-second read; built on the course template at 48 × 36 in, with the guide's minimum type sizes; strong contrast; every distinction carried in two channels (a label or pattern, never colour alone); each figure carries alt text in the file; no template guidance or EXAMPLE material left.</t>
+          <t>9–10 pts: A clear reading order: the finding is found in seconds, and the question, result, and boundary in a ninety-second read; built on the course template at 34 × 22.5 in, with the guide's minimum type sizes; strong contrast; every distinction carried in two channels (a label or pattern, never colour alone); each figure carries alt text in the file; no template guidance or EXAMPLE material left.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: D87 rubric — research design & methodology criterion (15), checks & verification 12, intro and closing notes dropped, table on one page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
+++ b/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
@@ -599,35 +599,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Data, provenance &amp; measurement</t>
+          <t>Research design &amp; methodology</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Data and measurement</t>
+          <t>Design: what your claim needs · Data and measurement · Methods</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>11–12 pts: Source and route can be identified (archive, URL or DOI, retrieval date, or collection protocol); observations and independent units are distinguished, with any grouping named; the time window is given; each key concept is tied to its measure with the main validity concern; missing data and their handling are reported; the permission or IRB determination is stated.</t>
+          <t>14–15 pts: The design and method fit the question: the data strategy (who or what was observed, how units were selected, sample size counted in independent units, time window) and the answer strategy (the comparison, estimator, or model, and how its uncertainty is computed) are stated and justified; the data source and route can be identified; each key concept is tied to its measure with the main validity concern; missing data and the permission or IRB determination are reported; what was declared in advance is kept apart from later changes.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>9–10 pts: The evidence is identifiable; one consequential detail is thin.</t>
+          <t>11–13 pts: Design and method are appropriate and clearly described; one justification or one consequential detail (selection, measurement, missing data) is thin.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>5–8 pts: Important provenance or measurement information is missing.</t>
+          <t>6–10 pts: Methods are named but not justified for this question, or the data, selection, or measurement are described too vaguely to judge the design.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>0–4 pts: The evidence cannot be identified, or a material permission problem is unresolved.</t>
+          <t>0–5 pts: No identifiable design or method, a method that cannot answer the question, or evidence that cannot be identified.</t>
         </is>
       </c>
       <c r="I4" s="2" t="n"/>
@@ -639,35 +639,35 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Analysis, checks &amp; verification</t>
+          <t>Checks &amp; verification</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Methods · Checks and verification · verification status line</t>
+          <t>Checks and verification · verification status line</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>14–15 pts: The analysis fits the design; what was declared in advance is kept apart from later changes, and each change is explained; the uncertainty method fits the data, computed at the level of the independent unit with any dependence named; at least one consequential robustness, sensitivity, or diagnostic check is reported with what it changed; the verification status is accurate and honestly labeled (an external cold run, or "solo proxy; external cold run pending").</t>
+          <t>11–12 pts: The uncertainty is computed at the level of the independent unit, with any dependence named; at least one consequential robustness, sensitivity, or diagnostic check is reported with what it changed; the verification status is accurate and honestly labeled (an external cold run, or "solo proxy; external cold run pending").</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>11–13 pts: Analysis and uncertainty are appropriate; the check or the verification account is thin.</t>
+          <t>9–10 pts: Uncertainty appropriate; the check or the verification account is thin.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>6–10 pts: A weak link between method and design, an uninformative check, or a verification claim the record does not support.</t>
+          <t>5–8 pts: An uninformative check, or a verification claim the record does not support.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>0–5 pts: A material analytical error, or a displayed result with no trace or that fails to reproduce.</t>
+          <t>0–4 pts: A material analytical error, or a displayed result with no trace or that fails to reproduce.</t>
         </is>
       </c>
       <c r="I5" s="2" t="n"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Analysis, checks &amp; verification</t>
+          <t>Checks &amp; verification</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Analysis, checks &amp; verification</t>
+          <t>Checks &amp; verification</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Analysis, checks &amp; verification</t>
+          <t>Checks &amp; verification</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Session auto commit (Claude Code Stop hook)
Automated commit + push at the end of a Claude Code session/turn.
Tracked changes only; docs/ re-rendered when content changed.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
+++ b/project/poster/Evidence_Driven_Research_Poster_Rubric.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>11–12 pts: The uncertainty is computed at the level of the independent unit, with any dependence named; at least one consequential robustness, sensitivity, or diagnostic check is reported with what it changed; the verification status is accurate and honestly labeled (an external cold run, or "solo proxy; external cold run pending").</t>
+          <t>11–12 pts: The uncertainty is computed at the level of the independent unit, with any dependence named; at least one consequential robustness, sensitivity, or diagnostic check is reported with what it changed; the verification status line says honestly what has been rerun, by whom and when, and what is still pending (an author rerun is never presented as independent reproduction).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>A displayed result or bound that materially fails to reproduce from the submitted package (documented rounding is not a failure)</t>
+          <t>A displayed result or bound that materially fails to reproduce when its traced notebook cell is rerun (documented rounding is not a failure)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>An author rerun presented as independent reproduction, or a solo proxy without its label</t>
+          <t>A verification status that claims more than was done, such as an author rerun presented as independent reproduction</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>